<commit_message>
Update: Novotel-February-2026 by superadmin
</commit_message>
<xml_diff>
--- a/Novotel-February-2026.xlsx
+++ b/Novotel-February-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2023031\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{834D72EA-451D-4C73-8B57-89CA029BA952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2764883F-7A96-434B-A750-4D6D932860BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{E82819E8-EFF0-4774-BA8F-CEEEEB2C50F6}"/>
   </bookViews>
@@ -657,7 +657,7 @@
       </c>
       <c r="G2" s="1">
         <f t="shared" ref="G2:G9" ca="1" si="0">TODAY()-RANDBETWEEN(365,365*5)</f>
-        <v>45747</v>
+        <v>44651</v>
       </c>
       <c r="H2">
         <v>77622</v>
@@ -719,7 +719,7 @@
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>22</v>
@@ -738,7 +738,7 @@
       </c>
       <c r="G3" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>44971</v>
+        <v>45347</v>
       </c>
       <c r="H3">
         <v>74250</v>
@@ -800,7 +800,7 @@
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B4" t="s">
         <v>22</v>
@@ -819,7 +819,7 @@
       </c>
       <c r="G4" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>44400</v>
+        <v>45639</v>
       </c>
       <c r="H4">
         <v>91399</v>
@@ -881,7 +881,7 @@
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
         <v>22</v>
@@ -900,7 +900,7 @@
       </c>
       <c r="G5" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>45439</v>
+        <v>45283</v>
       </c>
       <c r="H5">
         <v>100198</v>
@@ -962,7 +962,7 @@
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
         <v>22</v>
@@ -981,7 +981,7 @@
       </c>
       <c r="G6" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>44847</v>
+        <v>44797</v>
       </c>
       <c r="H6">
         <v>93482</v>
@@ -1043,7 +1043,7 @@
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
         <v>22</v>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="G7" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>44783</v>
+        <v>45642</v>
       </c>
       <c r="H7">
         <v>96107</v>
@@ -1124,7 +1124,7 @@
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
         <v>22</v>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="G8" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>45500</v>
+        <v>45064</v>
       </c>
       <c r="H8">
         <v>86027</v>
@@ -1205,7 +1205,7 @@
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
         <v>22</v>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="G9" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>44810</v>
+        <v>44804</v>
       </c>
       <c r="H9">
         <v>99500</v>

</xml_diff>